<commit_message>
Updated data for livestock
</commit_message>
<xml_diff>
--- a/data-preprocessing/rpc-footprints/6 - Wild foods/Wild foods.xlsx
+++ b/data-preprocessing/rpc-footprints/6 - Wild foods/Wild foods.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wilhelmwanecek/dev/safad/data-preprocessing/rpc-footprints/6 - Wild foods/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4020005A-EAE1-424A-93C8-CFB0D7559527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D27CD61-492A-6946-943C-24A6728E3E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="29400" yWindow="-21000" windowWidth="38400" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="143">
   <si>
     <t>A.06.03.001</t>
   </si>
@@ -462,6 +462,9 @@
   </si>
   <si>
     <t>21170.02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    </t>
   </si>
 </sst>
 </file>
@@ -4223,7 +4226,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76D1EA37-E052-405D-B3CF-60804D779B0E}">
-  <dimension ref="A1:AR11"/>
+  <dimension ref="A1:AR60"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="22.5" customWidth="1"/>
@@ -5896,6 +5899,11 @@
       </c>
     </row>
     <row r="11" spans="1:44" s="21" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="60" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F60" t="s">
+        <v>142</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
Updated wild data: RoW approximated as Sweden
</commit_message>
<xml_diff>
--- a/data-preprocessing/rpc-footprints/6 - Wild foods/Wild foods.xlsx
+++ b/data-preprocessing/rpc-footprints/6 - Wild foods/Wild foods.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wilhelmwanecek/dev/safad/data-preprocessing/rpc-footprints/6 - Wild foods/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D27CD61-492A-6946-943C-24A6728E3E3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C77E1040-29EB-9949-9572-4A0A6B7E8854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="29400" yWindow="-21000" windowWidth="38400" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="3" r:id="rId1"/>
     <sheet name="Wild foods" sheetId="4" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="146">
   <si>
     <t>A.06.03.001</t>
   </si>
@@ -464,7 +465,16 @@
     <t>21170.02</t>
   </si>
   <si>
-    <t xml:space="preserve">    </t>
+    <t>Rest of World</t>
+  </si>
+  <si>
+    <t>RoW</t>
+  </si>
+  <si>
+    <t>direct_values</t>
+  </si>
+  <si>
+    <t>N/P/Diesel</t>
   </si>
 </sst>
 </file>
@@ -4226,7 +4236,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76D1EA37-E052-405D-B3CF-60804D779B0E}">
-  <dimension ref="A1:AR60"/>
+  <dimension ref="A1:AS19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="22.5" customWidth="1"/>
@@ -4234,7 +4244,7 @@
     <col min="44" max="44" width="8.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44" s="21" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:45" s="21" customFormat="1" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="21" t="s">
         <v>112</v>
       </c>
@@ -4367,8 +4377,11 @@
       <c r="AR1" s="21" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="2" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS1" s="21" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="2" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>115</v>
       </c>
@@ -4537,8 +4550,11 @@
         <f>INFO!AR83</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>119</v>
       </c>
@@ -4707,8 +4723,11 @@
         <f>INFO!AR83</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="4" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>122</v>
       </c>
@@ -4877,8 +4896,11 @@
         <f>INFO!AR83</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS4" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="5" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -5047,8 +5069,11 @@
         <f>INFO!AR68</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS5" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -5217,8 +5242,11 @@
         <f>INFO!AR29</f>
         <v>3.977235735190196E-5</v>
       </c>
-    </row>
-    <row r="7" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="7" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>129</v>
       </c>
@@ -5387,8 +5415,11 @@
         <f>INFO!AR83</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS7" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="8" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -5557,8 +5588,11 @@
         <f>INFO!AR68</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS8" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="9" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>134</v>
       </c>
@@ -5727,8 +5761,11 @@
         <f>INFO!AR83</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="AS9" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="10" spans="1:45" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -5897,15 +5934,1551 @@
         <f>INFO!AR68</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:44" s="21" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="60" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F60" t="s">
+      <c r="AS10" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="11" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>115</v>
+      </c>
+      <c r="B11" t="s">
+        <v>116</v>
+      </c>
+      <c r="C11" t="s">
+        <v>117</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="E11" t="s">
+        <v>118</v>
+      </c>
+      <c r="F11" t="s">
+        <v>4</v>
+      </c>
+      <c r="G11" t="s">
         <v>142</v>
+      </c>
+      <c r="H11" t="s">
+        <v>143</v>
+      </c>
+      <c r="I11">
+        <f>I2</f>
+        <v>1.26</v>
+      </c>
+      <c r="J11">
+        <f t="shared" ref="J11:AR11" si="0">J2</f>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="K11">
+        <f t="shared" si="0"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="L11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <f t="shared" si="0"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="N11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Q11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="R11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="S11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="U11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="V11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="W11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="X11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Y11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="Z11">
+        <f t="shared" si="0"/>
+        <v>1.26</v>
+      </c>
+      <c r="AA11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AB11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AC11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AD11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AE11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AF11">
+        <f t="shared" si="0"/>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="AG11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AH11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AI11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AJ11">
+        <f t="shared" si="0"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="AK11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AL11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AM11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AN11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AO11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AP11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="AQ11">
+        <f t="shared" si="0"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="AR11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>119</v>
+      </c>
+      <c r="B12" t="s">
+        <v>120</v>
+      </c>
+      <c r="C12" t="s">
+        <v>121</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="E12" t="s">
+        <v>118</v>
+      </c>
+      <c r="F12" t="s">
+        <v>4</v>
+      </c>
+      <c r="G12" t="s">
+        <v>142</v>
+      </c>
+      <c r="H12" t="s">
+        <v>143</v>
+      </c>
+      <c r="I12">
+        <f t="shared" ref="I12:AR12" si="1">I3</f>
+        <v>1.26</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="1"/>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="K12">
+        <f t="shared" si="1"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="L12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <f t="shared" si="1"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="N12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="O12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="P12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Q12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="R12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="S12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="U12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="V12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="W12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="X12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Y12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="Z12">
+        <f t="shared" si="1"/>
+        <v>1.26</v>
+      </c>
+      <c r="AA12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AB12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AC12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AD12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AE12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AF12">
+        <f t="shared" si="1"/>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="AG12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AH12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AI12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AJ12">
+        <f t="shared" si="1"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="AK12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AL12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AM12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AN12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AO12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AP12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="AQ12">
+        <f t="shared" si="1"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="AR12">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>122</v>
+      </c>
+      <c r="B13" t="s">
+        <v>123</v>
+      </c>
+      <c r="C13" t="s">
+        <v>124</v>
+      </c>
+      <c r="D13" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="E13" t="s">
+        <v>118</v>
+      </c>
+      <c r="F13" t="s">
+        <v>4</v>
+      </c>
+      <c r="G13" t="s">
+        <v>142</v>
+      </c>
+      <c r="H13" t="s">
+        <v>143</v>
+      </c>
+      <c r="I13">
+        <f t="shared" ref="I13:AR13" si="2">I4</f>
+        <v>1.26</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="2"/>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="K13">
+        <f t="shared" si="2"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="L13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <f t="shared" si="2"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="N13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="P13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Q13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="R13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="S13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="T13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="U13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="V13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="W13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="X13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Y13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="Z13">
+        <f t="shared" si="2"/>
+        <v>1.26</v>
+      </c>
+      <c r="AA13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AB13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AC13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AD13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AE13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AF13">
+        <f t="shared" si="2"/>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="AG13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AH13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AI13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AJ13">
+        <f t="shared" si="2"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="AK13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AL13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AM13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AN13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AO13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AP13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="AQ13">
+        <f t="shared" si="2"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="AR13">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>2</v>
+      </c>
+      <c r="B14" t="s">
+        <v>125</v>
+      </c>
+      <c r="C14" t="s">
+        <v>126</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="E14" t="s">
+        <v>118</v>
+      </c>
+      <c r="F14" t="s">
+        <v>4</v>
+      </c>
+      <c r="G14" t="s">
+        <v>142</v>
+      </c>
+      <c r="H14" t="s">
+        <v>143</v>
+      </c>
+      <c r="I14">
+        <f t="shared" ref="I14:AR14" si="3">I5</f>
+        <v>24.344999999999999</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="3"/>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="K14">
+        <f t="shared" si="3"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="L14">
+        <f t="shared" si="3"/>
+        <v>0.85499999999999998</v>
+      </c>
+      <c r="M14">
+        <f t="shared" si="3"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="N14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="P14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="Q14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="R14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="S14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="T14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="U14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="V14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="W14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="X14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="Y14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="Z14">
+        <f t="shared" si="3"/>
+        <v>1.26</v>
+      </c>
+      <c r="AA14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AB14">
+        <f t="shared" si="3"/>
+        <v>23.085000000000001</v>
+      </c>
+      <c r="AC14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AD14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AE14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AF14">
+        <f t="shared" si="3"/>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="AG14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AH14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AI14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AJ14">
+        <f t="shared" si="3"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="AK14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AL14">
+        <f t="shared" si="3"/>
+        <v>0.85499999999999998</v>
+      </c>
+      <c r="AM14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AN14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AO14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AP14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="AQ14">
+        <f t="shared" si="3"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="AR14">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B15" t="s">
+        <v>127</v>
+      </c>
+      <c r="C15" t="s">
+        <v>128</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="E15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F15" t="s">
+        <v>4</v>
+      </c>
+      <c r="G15" t="s">
+        <v>142</v>
+      </c>
+      <c r="H15" t="s">
+        <v>143</v>
+      </c>
+      <c r="I15">
+        <f t="shared" ref="I15:AR15" si="4">I6</f>
+        <v>1.44</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="4"/>
+        <v>1.2933019622210329</v>
+      </c>
+      <c r="K15">
+        <f t="shared" si="4"/>
+        <v>6.2365945179634387E-4</v>
+      </c>
+      <c r="L15">
+        <f t="shared" si="4"/>
+        <v>7.0896838677521367E-4</v>
+      </c>
+      <c r="M15">
+        <f t="shared" si="4"/>
+        <v>3.9916058488097196E-4</v>
+      </c>
+      <c r="N15">
+        <f t="shared" si="4"/>
+        <v>0.54668896678386059</v>
+      </c>
+      <c r="O15">
+        <f t="shared" si="4"/>
+        <v>8.3643411917930597E-3</v>
+      </c>
+      <c r="P15">
+        <f t="shared" si="4"/>
+        <v>7.6536455349740333E-4</v>
+      </c>
+      <c r="Q15">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="R15">
+        <f t="shared" si="4"/>
+        <v>4.0454983542005524E-2</v>
+      </c>
+      <c r="S15">
+        <f t="shared" si="4"/>
+        <v>1.118595671518895E-14</v>
+      </c>
+      <c r="T15">
+        <f t="shared" si="4"/>
+        <v>5.0850679959101724E-4</v>
+      </c>
+      <c r="U15">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="V15">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="W15">
+        <f t="shared" si="4"/>
+        <v>4.2286996710240062E-2</v>
+      </c>
+      <c r="X15">
+        <f t="shared" si="4"/>
+        <v>1.0721917226493825E-2</v>
+      </c>
+      <c r="Y15">
+        <f t="shared" si="4"/>
+        <v>7.3679808690266704E-2</v>
+      </c>
+      <c r="Z15">
+        <f t="shared" si="4"/>
+        <v>2.3311277372999411E-2</v>
+      </c>
+      <c r="AA15">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AB15">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AC15">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AD15">
+        <f t="shared" si="4"/>
+        <v>2.624001350053411E-2</v>
+      </c>
+      <c r="AE15">
+        <f t="shared" si="4"/>
+        <v>9.6076759089496044E-3</v>
+      </c>
+      <c r="AF15">
+        <f t="shared" si="4"/>
+        <v>1.2574542728115492</v>
+      </c>
+      <c r="AG15">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AH15">
+        <f t="shared" si="4"/>
+        <v>3.3011233069633681E-5</v>
+      </c>
+      <c r="AI15">
+        <f t="shared" si="4"/>
+        <v>3.3804785605563428E-5</v>
+      </c>
+      <c r="AJ15">
+        <f t="shared" si="4"/>
+        <v>5.5684343312114659E-4</v>
+      </c>
+      <c r="AK15">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AL15">
+        <f t="shared" si="4"/>
+        <v>7.0896838677521367E-4</v>
+      </c>
+      <c r="AM15">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="AN15">
+        <f t="shared" si="4"/>
+        <v>5.5176734301212027E-5</v>
+      </c>
+      <c r="AO15">
+        <f t="shared" si="4"/>
+        <v>3.9142383332757652E-7</v>
+      </c>
+      <c r="AP15">
+        <f t="shared" si="4"/>
+        <v>2.6988940912185655E-4</v>
+      </c>
+      <c r="AQ15">
+        <f t="shared" si="4"/>
+        <v>3.3930660272673784E-5</v>
+      </c>
+      <c r="AR15">
+        <f t="shared" si="4"/>
+        <v>3.977235735190196E-5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:45" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>129</v>
+      </c>
+      <c r="B16" t="s">
+        <v>130</v>
+      </c>
+      <c r="C16" t="s">
+        <v>131</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="E16" t="s">
+        <v>118</v>
+      </c>
+      <c r="F16" t="s">
+        <v>4</v>
+      </c>
+      <c r="G16" t="s">
+        <v>142</v>
+      </c>
+      <c r="H16" t="s">
+        <v>143</v>
+      </c>
+      <c r="I16">
+        <f t="shared" ref="I16:AR16" si="5">I7</f>
+        <v>1.26</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="5"/>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="K16">
+        <f t="shared" si="5"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="L16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="M16">
+        <f t="shared" si="5"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="N16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="O16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="P16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Q16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="R16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="S16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="T16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="V16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="W16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="X16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Y16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="Z16">
+        <f t="shared" si="5"/>
+        <v>1.26</v>
+      </c>
+      <c r="AA16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AB16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AC16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AD16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AE16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AF16">
+        <f t="shared" si="5"/>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="AG16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AH16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AI16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AJ16">
+        <f t="shared" si="5"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="AK16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AL16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AM16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AN16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AO16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AP16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="AQ16">
+        <f t="shared" si="5"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="AR16">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" t="s">
+        <v>132</v>
+      </c>
+      <c r="C17" t="s">
+        <v>133</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="E17" t="s">
+        <v>118</v>
+      </c>
+      <c r="F17" t="s">
+        <v>4</v>
+      </c>
+      <c r="G17" t="s">
+        <v>142</v>
+      </c>
+      <c r="H17" t="s">
+        <v>143</v>
+      </c>
+      <c r="I17">
+        <f t="shared" ref="I17:AR17" si="6">I8</f>
+        <v>24.344999999999999</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="6"/>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="K17">
+        <f t="shared" si="6"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="L17">
+        <f t="shared" si="6"/>
+        <v>0.85499999999999998</v>
+      </c>
+      <c r="M17">
+        <f t="shared" si="6"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="N17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="O17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="P17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="Q17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="R17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="S17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="T17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="U17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="V17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="W17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="X17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="Y17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="Z17">
+        <f t="shared" si="6"/>
+        <v>1.26</v>
+      </c>
+      <c r="AA17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="AB17">
+        <f t="shared" si="6"/>
+        <v>23.085000000000001</v>
+      </c>
+      <c r="AC17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="AD17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="AE17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="AF17">
+        <f t="shared" si="6"/>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="AG17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="AH17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="AI17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="AJ17">
+        <f t="shared" si="6"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="AK17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="AL17">
+        <f t="shared" si="6"/>
+        <v>0.85499999999999998</v>
+      </c>
+      <c r="AM17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="AN17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="AO17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="AP17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="AQ17">
+        <f t="shared" si="6"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="AR17">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>134</v>
+      </c>
+      <c r="B18" t="s">
+        <v>135</v>
+      </c>
+      <c r="C18" t="s">
+        <v>136</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="E18" t="s">
+        <v>118</v>
+      </c>
+      <c r="F18" t="s">
+        <v>4</v>
+      </c>
+      <c r="G18" t="s">
+        <v>142</v>
+      </c>
+      <c r="H18" t="s">
+        <v>143</v>
+      </c>
+      <c r="I18">
+        <f t="shared" ref="I18:AR18" si="7">I9</f>
+        <v>1.26</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="7"/>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="K18">
+        <f t="shared" si="7"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="L18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <f t="shared" si="7"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="N18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="O18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="P18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Q18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="R18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="S18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="T18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="U18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="V18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="W18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="X18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Y18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Z18">
+        <f t="shared" si="7"/>
+        <v>1.26</v>
+      </c>
+      <c r="AA18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AB18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AC18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AD18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AE18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AF18">
+        <f t="shared" si="7"/>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="AG18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AH18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AI18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AJ18">
+        <f t="shared" si="7"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="AK18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AL18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AM18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AN18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AO18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AP18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="AQ18">
+        <f t="shared" si="7"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="AR18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>1</v>
+      </c>
+      <c r="B19" t="s">
+        <v>137</v>
+      </c>
+      <c r="C19" t="s">
+        <v>138</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>141</v>
+      </c>
+      <c r="E19" t="s">
+        <v>118</v>
+      </c>
+      <c r="F19" t="s">
+        <v>4</v>
+      </c>
+      <c r="G19" t="s">
+        <v>142</v>
+      </c>
+      <c r="H19" t="s">
+        <v>143</v>
+      </c>
+      <c r="I19">
+        <f t="shared" ref="I19:AR19" si="8">I10</f>
+        <v>24.344999999999999</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="8"/>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="K19">
+        <f t="shared" si="8"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="L19">
+        <f t="shared" si="8"/>
+        <v>0.85499999999999998</v>
+      </c>
+      <c r="M19">
+        <f t="shared" si="8"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="N19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="Q19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="R19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="S19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="T19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="V19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="W19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="X19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="Y19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="Z19">
+        <f t="shared" si="8"/>
+        <v>1.26</v>
+      </c>
+      <c r="AA19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AB19">
+        <f t="shared" si="8"/>
+        <v>23.085000000000001</v>
+      </c>
+      <c r="AC19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AD19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AE19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AF19">
+        <f t="shared" si="8"/>
+        <v>1.2346453096108738</v>
+      </c>
+      <c r="AG19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AH19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AI19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AJ19">
+        <f t="shared" si="8"/>
+        <v>5.4690624028205586E-4</v>
+      </c>
+      <c r="AK19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AL19">
+        <f t="shared" si="8"/>
+        <v>0.85499999999999998</v>
+      </c>
+      <c r="AM19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AN19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AO19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AP19">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="AQ19">
+        <f t="shared" si="8"/>
+        <v>3.3175400837805351E-5</v>
+      </c>
+      <c r="AR19">
+        <f t="shared" si="8"/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C207F371-DEAC-644E-8D4E-A0A0D7D24000}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Bugfix: Fix colname for direct values of wild foods
</commit_message>
<xml_diff>
--- a/data-preprocessing/rpc-footprints/6 - Wild foods/Wild foods.xlsx
+++ b/data-preprocessing/rpc-footprints/6 - Wild foods/Wild foods.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/wilhelmwanecek/dev/safad/data-preprocessing/rpc-footprints/6 - Wild foods/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C77E1040-29EB-9949-9572-4A0A6B7E8854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1057439A-2391-9740-AB94-7B17B26F3BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="29400" yWindow="-21000" windowWidth="38400" windowHeight="21000" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -471,10 +471,10 @@
     <t>RoW</t>
   </si>
   <si>
-    <t>direct_values</t>
-  </si>
-  <si>
     <t>N/P/Diesel</t>
+  </si>
+  <si>
+    <t>Direct Values (N-P-Diesel)</t>
   </si>
 </sst>
 </file>
@@ -4378,7 +4378,7 @@
         <v>98</v>
       </c>
       <c r="AS1" s="21" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:45" x14ac:dyDescent="0.2">
@@ -4551,7 +4551,7 @@
         <v>0</v>
       </c>
       <c r="AS2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:45" x14ac:dyDescent="0.2">
@@ -4724,7 +4724,7 @@
         <v>0</v>
       </c>
       <c r="AS3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:45" x14ac:dyDescent="0.2">
@@ -4897,7 +4897,7 @@
         <v>0</v>
       </c>
       <c r="AS4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="5" spans="1:45" x14ac:dyDescent="0.2">
@@ -5070,7 +5070,7 @@
         <v>0</v>
       </c>
       <c r="AS5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:45" x14ac:dyDescent="0.2">
@@ -5243,7 +5243,7 @@
         <v>3.977235735190196E-5</v>
       </c>
       <c r="AS6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:45" x14ac:dyDescent="0.2">
@@ -5416,7 +5416,7 @@
         <v>0</v>
       </c>
       <c r="AS7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="8" spans="1:45" x14ac:dyDescent="0.2">
@@ -5589,7 +5589,7 @@
         <v>0</v>
       </c>
       <c r="AS8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:45" x14ac:dyDescent="0.2">
@@ -5762,7 +5762,7 @@
         <v>0</v>
       </c>
       <c r="AS9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:45" x14ac:dyDescent="0.2">
@@ -5935,7 +5935,7 @@
         <v>0</v>
       </c>
       <c r="AS10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="11" spans="1:45" x14ac:dyDescent="0.2">

</xml_diff>